<commit_message>
updated with 3-2 running example
</commit_message>
<xml_diff>
--- a/LAFExamples/analysis/diagnosis-scores-trust.xlsx
+++ b/LAFExamples/analysis/diagnosis-scores-trust.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="33">
   <si>
     <t>Time</t>
   </si>
@@ -26,52 +26,61 @@
     <t>#Arg-</t>
   </si>
   <si>
-    <t>L9: Headache</t>
-  </si>
-  <si>
-    <t>L5: Fever</t>
-  </si>
-  <si>
-    <t>L14: Runny nose</t>
-  </si>
-  <si>
-    <t>L15: Sore throat</t>
-  </si>
-  <si>
-    <t>L4: COVID test is negative</t>
-  </si>
-  <si>
-    <t>L3: No red spots on the back of the roof of the mouth</t>
-  </si>
-  <si>
-    <t>L7: No known allergies</t>
-  </si>
-  <si>
-    <t>L10: Allergies</t>
-  </si>
-  <si>
-    <t>L11: Flu</t>
-  </si>
-  <si>
-    <t>L6: Sinus Infection</t>
-  </si>
-  <si>
-    <t>L2: COVID-19</t>
-  </si>
-  <si>
-    <t>L13: Common Cold</t>
+    <t>L5: Headache</t>
+  </si>
+  <si>
+    <t>L11: Runny nose</t>
+  </si>
+  <si>
+    <t>L15: No known allergies</t>
+  </si>
+  <si>
+    <t>L1: Fever</t>
+  </si>
+  <si>
+    <t>L0: Sore throat</t>
+  </si>
+  <si>
+    <t>L12: No red spots on the back of the roof of the mouth</t>
+  </si>
+  <si>
+    <t>L9: COVID test is negative</t>
+  </si>
+  <si>
+    <t>L6: Allergies</t>
+  </si>
+  <si>
+    <t>L18: Common Cold</t>
+  </si>
+  <si>
+    <t>L16: Sinus Infection</t>
+  </si>
+  <si>
+    <t>L2: Flu</t>
+  </si>
+  <si>
+    <t>L3: COVID-19</t>
+  </si>
+  <si>
+    <t>L13: Introduction of fever and sore throat eliminates  common cold</t>
+  </si>
+  <si>
+    <t>L7: Introduction of fever and sore throat eliminates  sinus infection</t>
   </si>
   <si>
     <t>L8: Strep Throat</t>
   </si>
   <si>
-    <t>L12: Strep throat causes red spots  on the back of the roof of the mouth</t>
-  </si>
-  <si>
-    <t>L0: Fever is not a common  symptom of the common cold</t>
-  </si>
-  <si>
-    <t>L1: Fever and sore throat are not common  symptoms of Sinus infection</t>
+    <t>L4: Strep throat causes red spots  on the back of the roof of the mouth</t>
+  </si>
+  <si>
+    <t>L14: Eliminating strep throat makes Flu or COVID more likely</t>
+  </si>
+  <si>
+    <t>L10: Common cold is still possible  but is less likely</t>
+  </si>
+  <si>
+    <t>L17: Sinus infection is still possible but is less likely</t>
   </si>
   <si>
     <t>Undercuts</t>
@@ -86,22 +95,22 @@
     <t>logAccumulator</t>
   </si>
   <si>
+    <t>[1.0]</t>
+  </si>
+  <si>
     <t>[]</t>
   </si>
   <si>
-    <t>[1.0, 1.0]</t>
-  </si>
-  <si>
-    <t>[1.0]</t>
+    <t>[1.0, 1.0, 0.5]</t>
+  </si>
+  <si>
+    <t>[0.5]</t>
   </si>
   <si>
     <t>Rebuttals</t>
   </si>
   <si>
-    <t>[0.5]</t>
-  </si>
-  <si>
-    <t>[0.33333334]</t>
+    <t>[0.25]</t>
   </si>
 </sst>
 </file>
@@ -384,18 +393,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:J18"/>
+  <dimension ref="A1:J21"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="5" max="5" width="8.07421875" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="11.51171875" customWidth="true" bestFit="true"/>
     <col min="8" max="8" width="5.609375" customWidth="true" bestFit="true"/>
     <col min="1" max="1" width="2.9296875" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="58.4453125" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="57.4453125" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="1.9296875" customWidth="true" bestFit="true"/>
     <col min="4" max="4" width="1.9296875" customWidth="true" bestFit="true"/>
     <col min="6" max="6" width="5.23046875" customWidth="true" bestFit="true"/>
     <col min="7" max="7" width="13.59765625" customWidth="true" bestFit="true"/>
-    <col min="9" max="9" width="11.63671875" customWidth="true" bestFit="true"/>
+    <col min="9" max="9" width="5.63671875" customWidth="true" bestFit="true"/>
     <col min="10" max="10" width="13.59765625" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
@@ -413,11 +422,11 @@
         <v>3</v>
       </c>
       <c r="E1" t="s" s="12">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="F1" s="0"/>
       <c r="H1" t="s" s="12">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="I1" s="0"/>
     </row>
@@ -426,22 +435,22 @@
       <c r="B2" s="0"/>
       <c r="C2" s="0"/>
       <c r="E2" t="s" s="13">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="F2" t="s" s="2">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="G2" t="s" s="2">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="H2" t="s" s="13">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="I2" t="s" s="2">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="J2" t="s" s="2">
-        <v>23</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3">
@@ -458,19 +467,19 @@
         <v>0.0</v>
       </c>
       <c r="E3" t="s" s="15">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F3" t="s" s="0">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="G3" t="n" s="5">
         <v>0.6931471824645996</v>
       </c>
       <c r="H3" t="s" s="15">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I3" t="s" s="0">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="J3" t="n" s="5">
         <v>0.28768208622932434</v>
@@ -490,19 +499,19 @@
         <v>0.0</v>
       </c>
       <c r="E4" t="s" s="15">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F4" t="s" s="0">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="G4" t="n" s="5">
         <v>0.6931471824645996</v>
       </c>
       <c r="H4" t="s" s="15">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I4" t="s" s="0">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="J4" t="n" s="5">
         <v>0.28768208622932434</v>
@@ -522,19 +531,19 @@
         <v>0.0</v>
       </c>
       <c r="E5" t="s" s="15">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F5" t="s" s="0">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="G5" t="n" s="5">
         <v>0.6931471824645996</v>
       </c>
       <c r="H5" t="s" s="15">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I5" t="s" s="0">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="J5" t="n" s="5">
         <v>0.28768208622932434</v>
@@ -554,19 +563,19 @@
         <v>0.0</v>
       </c>
       <c r="E6" t="s" s="15">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F6" t="s" s="0">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="G6" t="n" s="5">
         <v>0.6931471824645996</v>
       </c>
       <c r="H6" t="s" s="15">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I6" t="s" s="0">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="J6" t="n" s="5">
         <v>0.28768208622932434</v>
@@ -586,19 +595,19 @@
         <v>0.0</v>
       </c>
       <c r="E7" t="s" s="15">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F7" t="s" s="0">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="G7" t="n" s="5">
         <v>0.6931471824645996</v>
       </c>
       <c r="H7" t="s" s="15">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I7" t="s" s="0">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="J7" t="n" s="5">
         <v>0.28768208622932434</v>
@@ -618,19 +627,19 @@
         <v>0.0</v>
       </c>
       <c r="E8" t="s" s="15">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F8" t="s" s="0">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="G8" t="n" s="5">
         <v>0.6931471824645996</v>
       </c>
       <c r="H8" t="s" s="15">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I8" t="s" s="0">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="J8" t="n" s="5">
         <v>0.28768208622932434</v>
@@ -650,19 +659,19 @@
         <v>0.0</v>
       </c>
       <c r="E9" t="s" s="15">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F9" t="s" s="0">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="G9" t="n" s="5">
         <v>0.6931471824645996</v>
       </c>
       <c r="H9" t="s" s="15">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I9" t="s" s="0">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="J9" t="n" s="5">
         <v>0.28768208622932434</v>
@@ -682,19 +691,19 @@
         <v>1.0</v>
       </c>
       <c r="E10" t="s" s="15">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F10" t="s" s="0">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G10" t="n" s="7">
         <v>0.0</v>
       </c>
       <c r="H10" t="s" s="15">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="I10" t="s" s="0">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="J10" t="n" s="7">
         <v>0.0</v>
@@ -708,28 +717,28 @@
         <v>12</v>
       </c>
       <c r="C11" t="n" s="0">
-        <v>2.0</v>
+        <v>1.0</v>
       </c>
       <c r="D11" t="n" s="0">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="E11" t="s" s="15">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="F11" t="s" s="0">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="G11" t="n" s="5">
-        <v>1.0986123085021973</v>
+        <v>0.28768208622932434</v>
       </c>
       <c r="H11" t="s" s="15">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="I11" t="s" s="0">
-        <v>29</v>
-      </c>
-      <c r="J11" t="n" s="5">
-        <v>0.4054650664329529</v>
+        <v>30</v>
+      </c>
+      <c r="J11" t="n" s="7">
+        <v>0.0</v>
       </c>
     </row>
     <row r="12">
@@ -746,19 +755,19 @@
         <v>1.0</v>
       </c>
       <c r="E12" t="s" s="15">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F12" t="s" s="0">
-        <v>26</v>
-      </c>
-      <c r="G12" t="n" s="7">
-        <v>0.0</v>
+        <v>30</v>
+      </c>
+      <c r="G12" t="n" s="5">
+        <v>0.28768208622932434</v>
       </c>
       <c r="H12" t="s" s="15">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="I12" t="s" s="0">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="J12" t="n" s="7">
         <v>0.0</v>
@@ -772,28 +781,28 @@
         <v>14</v>
       </c>
       <c r="C13" t="n" s="0">
-        <v>2.0</v>
+        <v>3.0</v>
       </c>
       <c r="D13" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="E13" t="s" s="15">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="F13" t="s" s="0">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="G13" t="n" s="5">
-        <v>0.40546509623527527</v>
+        <v>1.2527629137039185</v>
       </c>
       <c r="H13" t="s" s="15">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I13" t="s" s="0">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="J13" t="n" s="5">
-        <v>0.11778300255537033</v>
+        <v>0.4700036346912384</v>
       </c>
     </row>
     <row r="14">
@@ -804,28 +813,28 @@
         <v>15</v>
       </c>
       <c r="C14" t="n" s="0">
-        <v>2.0</v>
+        <v>3.0</v>
       </c>
       <c r="D14" t="n" s="0">
         <v>1.0</v>
       </c>
       <c r="E14" t="s" s="15">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="F14" t="s" s="0">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G14" t="n" s="5">
-        <v>0.40546509623527527</v>
+        <v>0.5596157908439636</v>
       </c>
       <c r="H14" t="s" s="15">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="I14" t="s" s="0">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="J14" t="n" s="5">
-        <v>0.11778300255537033</v>
+        <v>0.18232156336307526</v>
       </c>
     </row>
     <row r="15">
@@ -836,89 +845,89 @@
         <v>16</v>
       </c>
       <c r="C15" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="D15" t="n" s="0">
         <v>1.0</v>
       </c>
       <c r="E15" t="s" s="15">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="F15" t="s" s="0">
-        <v>26</v>
-      </c>
-      <c r="G15" t="n" s="7">
-        <v>0.0</v>
+        <v>27</v>
+      </c>
+      <c r="G15" t="n" s="6">
+        <v>-0.6931471824645996</v>
       </c>
       <c r="H15" t="s" s="15">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="I15" t="s" s="0">
-        <v>28</v>
-      </c>
-      <c r="J15" t="n" s="7">
-        <v>0.0</v>
+        <v>27</v>
+      </c>
+      <c r="J15" t="n" s="6">
+        <v>-0.28768208622932434</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n" s="8">
-        <v>7.0</v>
-      </c>
-      <c r="B16" t="s" s="11">
+        <v>5.0</v>
+      </c>
+      <c r="B16" t="s" s="10">
         <v>17</v>
       </c>
       <c r="C16" t="n" s="0">
         <v>0.0</v>
       </c>
       <c r="D16" t="n" s="0">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="E16" t="s" s="15">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="F16" t="s" s="0">
-        <v>24</v>
-      </c>
-      <c r="G16" t="n" s="7">
-        <v>0.0</v>
+        <v>27</v>
+      </c>
+      <c r="G16" t="n" s="6">
+        <v>-0.6931471824645996</v>
       </c>
       <c r="H16" t="s" s="15">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="I16" t="s" s="0">
-        <v>26</v>
-      </c>
-      <c r="J16" t="n" s="7">
-        <v>0.0</v>
+        <v>27</v>
+      </c>
+      <c r="J16" t="n" s="6">
+        <v>-0.28768208622932434</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n" s="8">
-        <v>13.0</v>
+        <v>5.0</v>
       </c>
       <c r="B17" t="s" s="10">
         <v>18</v>
       </c>
       <c r="C17" t="n" s="0">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="D17" t="n" s="0">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="E17" t="s" s="15">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="F17" t="s" s="0">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="G17" t="n" s="7">
         <v>0.0</v>
       </c>
       <c r="H17" t="s" s="15">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="I17" t="s" s="0">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="J17" t="n" s="7">
         <v>0.0</v>
@@ -926,33 +935,129 @@
     </row>
     <row r="18">
       <c r="A18" t="n" s="8">
+        <v>7.0</v>
+      </c>
+      <c r="B18" t="s" s="11">
+        <v>19</v>
+      </c>
+      <c r="C18" t="n" s="0">
+        <v>0.0</v>
+      </c>
+      <c r="D18" t="n" s="0">
+        <v>0.0</v>
+      </c>
+      <c r="E18" t="s" s="15">
+        <v>28</v>
+      </c>
+      <c r="F18" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="G18" t="n" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="H18" t="s" s="15">
+        <v>27</v>
+      </c>
+      <c r="I18" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="J18" t="n" s="7">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n" s="8">
+        <v>9.0</v>
+      </c>
+      <c r="B19" t="s" s="10">
+        <v>20</v>
+      </c>
+      <c r="C19" t="n" s="0">
+        <v>0.0</v>
+      </c>
+      <c r="D19" t="n" s="0">
+        <v>0.0</v>
+      </c>
+      <c r="E19" t="s" s="15">
+        <v>28</v>
+      </c>
+      <c r="F19" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="G19" t="n" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="H19" t="s" s="15">
+        <v>27</v>
+      </c>
+      <c r="I19" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="J19" t="n" s="7">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n" s="8">
+        <v>13.0</v>
+      </c>
+      <c r="B20" t="s" s="10">
+        <v>21</v>
+      </c>
+      <c r="C20" t="n" s="0">
+        <v>0.0</v>
+      </c>
+      <c r="D20" t="n" s="0">
+        <v>0.0</v>
+      </c>
+      <c r="E20" t="s" s="15">
+        <v>28</v>
+      </c>
+      <c r="F20" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="G20" t="n" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="H20" t="s" s="15">
+        <v>27</v>
+      </c>
+      <c r="I20" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="J20" t="n" s="7">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n" s="8">
         <v>15.0</v>
       </c>
-      <c r="B18" t="s" s="10">
-        <v>19</v>
-      </c>
-      <c r="C18" t="n" s="0">
-        <v>0.0</v>
-      </c>
-      <c r="D18" t="n" s="0">
-        <v>0.0</v>
-      </c>
-      <c r="E18" t="s" s="15">
-        <v>24</v>
-      </c>
-      <c r="F18" t="s" s="0">
-        <v>24</v>
-      </c>
-      <c r="G18" t="n" s="7">
-        <v>0.0</v>
-      </c>
-      <c r="H18" t="s" s="15">
-        <v>26</v>
-      </c>
-      <c r="I18" t="s" s="0">
-        <v>26</v>
-      </c>
-      <c r="J18" t="n" s="7">
+      <c r="B21" t="s" s="10">
+        <v>22</v>
+      </c>
+      <c r="C21" t="n" s="0">
+        <v>0.0</v>
+      </c>
+      <c r="D21" t="n" s="0">
+        <v>0.0</v>
+      </c>
+      <c r="E21" t="s" s="15">
+        <v>28</v>
+      </c>
+      <c r="F21" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="G21" t="n" s="7">
+        <v>0.0</v>
+      </c>
+      <c r="H21" t="s" s="15">
+        <v>27</v>
+      </c>
+      <c r="I21" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="J21" t="n" s="7">
         <v>0.0</v>
       </c>
     </row>

</xml_diff>